<commit_message>
ABS ARI March 2026 update
</commit_message>
<xml_diff>
--- a/Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e).xlsx
+++ b/Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="33">
   <si>
     <t>Acute respiratory infection associated deaths, 2024-2026 (a)(b)(c)(d)(e)</t>
   </si>
@@ -97,7 +97,7 @@
     <t>a. Includes acute respiratory disease death registrations only. Numbers will differ to disease surveillance systems.</t>
   </si>
   <si>
-    <t>b. Includes all deaths (both doctor and coroner certified) that occurred and were registered by 28 February 2026.</t>
+    <t>b. Includes all deaths (both doctor and coroner certified) that occurred and were registered by 31 March 2026.</t>
   </si>
   <si>
     <t>c. All deaths involving COVID-19 in this report have been coded to ICD-10 codes U07.1-U07.2, U10.9 or U09.9. All deaths involving influenza have been coded to J09-J11. All deaths involving RSV have been coded to J12.1, J20.5, J21.0, B97.4.</t>
@@ -109,7 +109,7 @@
     <t>e. Refer to the methodology for more information regarding the data in this table.</t>
   </si>
   <si>
-    <t>Source: Australian Bureau of Statistics, Deaths due to acute respiratory infections in Australia February 2026</t>
+    <t>Source: Australian Bureau of Statistics, Deaths due to acute respiratory infections in Australia March 2026</t>
   </si>
 </sst>
 </file>
@@ -572,25 +572,25 @@
         <v>876</v>
       </c>
       <c r="H3" s="2">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="I3" s="2">
         <v>392</v>
       </c>
       <c r="J3" s="2">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="K3" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="L3" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="M3" s="2">
         <v>300</v>
       </c>
       <c r="N3" s="2">
-        <v>5111</v>
+        <v>5120</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -616,7 +616,7 @@
         <v>122</v>
       </c>
       <c r="H4" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I4" s="2">
         <v>272</v>
@@ -634,7 +634,7 @@
         <v>16</v>
       </c>
       <c r="N4" s="2">
-        <v>1045</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -686,7 +686,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C6" s="2">
         <v>168</v>
@@ -698,7 +698,7 @@
         <v>129</v>
       </c>
       <c r="F6" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G6" s="2">
         <v>359</v>
@@ -707,7 +707,7 @@
         <v>360</v>
       </c>
       <c r="I6" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J6" s="2">
         <v>152</v>
@@ -719,10 +719,10 @@
         <v>56</v>
       </c>
       <c r="M6" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N6" s="2">
-        <v>2172</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -745,28 +745,28 @@
         <v>80</v>
       </c>
       <c r="G7" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H7" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I7" s="2">
         <v>300</v>
       </c>
       <c r="J7" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K7" s="2">
         <v>125</v>
       </c>
       <c r="L7" s="2">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M7" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N7" s="2">
-        <v>1738</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -807,10 +807,10 @@
         <v>24</v>
       </c>
       <c r="M8" s="2">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="N8" s="2">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -818,13 +818,13 @@
         <v>21</v>
       </c>
       <c r="B9" s="2">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>22</v>
+        <v>45</v>
+      </c>
+      <c r="D9" s="2">
+        <v>18</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
@@ -854,7 +854,7 @@
         <v>22</v>
       </c>
       <c r="N9" s="2">
-        <v>90</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -862,13 +862,13 @@
         <v>23</v>
       </c>
       <c r="B10" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C10" s="2">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+      <c r="D10" s="2">
+        <v>9</v>
       </c>
       <c r="E10" t="s">
         <v>22</v>
@@ -898,7 +898,7 @@
         <v>22</v>
       </c>
       <c r="N10" s="2">
-        <v>112</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -906,13 +906,13 @@
         <v>24</v>
       </c>
       <c r="B11" s="2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2">
-        <v>2</v>
-      </c>
-      <c r="D11" t="s">
-        <v>22</v>
+        <v>16</v>
+      </c>
+      <c r="D11" s="2">
+        <v>17</v>
       </c>
       <c r="E11" t="s">
         <v>22</v>
@@ -942,7 +942,7 @@
         <v>22</v>
       </c>
       <c r="N11" s="2">
-        <v>24</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>